<commit_message>
Let protected sheets take input in the cells they leave unlocked, and hide formulas they protect
</commit_message>
<xml_diff>
--- a/tests/corpus/templates.xlsx
+++ b/tests/corpus/templates.xlsx
@@ -199,7 +199,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyProtection="1">
@@ -211,8 +211,11 @@
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -626,10 +629,10 @@
       <c r="C2">
         <v>120</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="7">
         <v>0.25</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="7">
         <f>[@Qty]*[@Price]</f>
         <v>30.0</v>
       </c>
@@ -647,10 +650,10 @@
       <c r="C3">
         <v>300</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="7">
         <v>0.1</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="7">
         <f>[@Qty]*[@Price]</f>
         <v>30.0</v>
       </c>
@@ -665,10 +668,10 @@
       <c r="C4">
         <v>15</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="7">
         <v>4.5</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="7">
         <f>[@Qty]*[@Price]</f>
         <v>67.5</v>
       </c>
@@ -683,10 +686,10 @@
       <c r="C5">
         <v>8</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="7">
         <v>12</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="7">
         <f>[@Qty]*[@Price]</f>
         <v>96.0</v>
       </c>
@@ -701,10 +704,10 @@
       <c r="C6">
         <v>40</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="7">
         <v>3.75</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="7">
         <f>[@Qty]*[@Price]</f>
         <v>150.0</v>
       </c>
@@ -717,7 +720,7 @@
         <f>SUBTOTAL(109,[Qty])</f>
         <v>483</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="7">
         <f>SUBTOTAL(109,[Total])</f>
         <v>373.5</v>
       </c>
@@ -795,7 +798,7 @@
       <c r="D3" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="7">
         <f>_xlfn.LET(net,SUM(Orders[Total]),rate,0.2,net*(1+rate))</f>
         <v>448.2</v>
       </c>

</xml_diff>

<commit_message>
Spill the results of dynamic array formulas into the cells around them, typed or from the file, recalculating as their inputs change and saving them as Excel does
</commit_message>
<xml_diff>
--- a/tests/corpus/templates.xlsx
+++ b/tests/corpus/templates.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>Purchase request</t>
   </si>
@@ -134,6 +134,15 @@
   </si>
   <si>
     <t>Hardware lines</t>
+  </si>
+  <si>
+    <t>From the Orders table</t>
+  </si>
+  <si>
+    <t>Grid</t>
+  </si>
+  <si>
+    <t>Doubled prices</t>
   </si>
 </sst>
 </file>
@@ -760,10 +769,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
@@ -773,8 +782,11 @@
       <c r="D1" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" cm="1" t="str">
         <f t="array" ref="A2:A4">_xlfn._xlws.SORT(_xlfn.UNIQUE(Orders[Category]))</f>
         <v>Electrical</v>
@@ -787,8 +799,18 @@
         <f t="array" ref="D2">_xlfn.XLOOKUP(MAX(Orders[Total]),Orders[Total],Orders[Item])</f>
         <v>Gloves</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="G2" cm="1">
+        <f t="array" ref="G2:I3">_xlfn.SEQUENCE(2,3)</f>
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -802,8 +824,17 @@
         <f>_xlfn.LET(net,SUM(Orders[Total]),rate,0.2,net*(1+rate))</f>
         <v>448.2</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -818,7 +849,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:9">
       <c r="D5" t="s">
         <v>30</v>
       </c>
@@ -826,10 +857,30 @@
         <f t="array" ref="E5:E6">_xlfn._xlws.FILTER(Orders[Item],Orders[Category]="Hardware")</f>
         <v>Bolts</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="G5" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
       <c r="E6" t="s">
         <v>13</v>
+      </c>
+      <c r="G6" s="7">
+        <f t="array" ref="G6:G8">Orders[Price]*2</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="G7" s="7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="G8" s="7">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>